<commit_message>
chore: refresh R1 verified workbook artifacts
</commit_message>
<xml_diff>
--- a/artifacts/ENG001-r1-synthetic-scenario.xlsx
+++ b/artifacts/ENG001-r1-synthetic-scenario.xlsx
@@ -12,7 +12,7 @@
     <sheet sheetId="6" name="Location Analysis" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="Provider Analysis" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="Service Line" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Collection Curves" state="visible" r:id="rId12"/>
+    <sheet sheetId="9" name="Recovery Analysis" state="visible" r:id="rId12"/>
     <sheet sheetId="10" name="Assumptions" state="visible" r:id="rId13"/>
     <sheet sheetId="11" name="Reconciliation" state="visible" r:id="rId14"/>
     <sheet sheetId="12" name="Findings" state="visible" r:id="rId15"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="131">
   <si>
     <t>Redwood Quality of Revenue Databook</t>
   </si>
@@ -52,21 +52,33 @@
     <t>Allowed amount</t>
   </si>
   <si>
+    <t>All cash</t>
+  </si>
+  <si>
+    <t>Allocated collections</t>
+  </si>
+  <si>
+    <t>Unapplied cash</t>
+  </si>
+  <si>
+    <t>Subsequent cash</t>
+  </si>
+  <si>
+    <t>Open A/R</t>
+  </si>
+  <si>
+    <t>Expected remaining cash</t>
+  </si>
+  <si>
+    <t>Realizable revenue</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
     <t>Observed cash</t>
   </si>
   <si>
-    <t>Open A/R</t>
-  </si>
-  <si>
-    <t>Expected remaining cash</t>
-  </si>
-  <si>
-    <t>Realizable revenue</t>
-  </si>
-  <si>
-    <t>Amount</t>
-  </si>
-  <si>
     <t>Cash event ID</t>
   </si>
   <si>
@@ -232,7 +244,7 @@
     <t>Authoritative editable recovery rates</t>
   </si>
   <si>
-    <t>Collection Curves!B2:B6</t>
+    <t>Recovery Analysis!B2:B6</t>
   </si>
   <si>
     <t>Important</t>
@@ -389,6 +401,21 @@
   </si>
   <si>
     <t>bf94986286656f63b92f66fc57c5412a219ec14a7e0fc6604d7aba34d9fd5fe2:3</t>
+  </si>
+  <si>
+    <t>general_ledger.csv</t>
+  </si>
+  <si>
+    <t>45aed22e980cb357ba709f0da96d3a033b7669da1e9ce3bff1fa9ef88da1044e</t>
+  </si>
+  <si>
+    <t>45aed22e980cb357ba709f0da96d3a033b7669da1e9ce3bff1fa9ef88da1044e:2</t>
+  </si>
+  <si>
+    <t>GLRecord</t>
+  </si>
+  <si>
+    <t>ENG001-GL-202606</t>
   </si>
 </sst>
 </file>
@@ -778,7 +805,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -844,7 +871,7 @@
         <v>10</v>
       </c>
       <c r="B9" s="1">
-        <v>15911.29</v>
+        <v>53205.59</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -852,7 +879,7 @@
         <v>11</v>
       </c>
       <c r="B10" s="1">
-        <f>SUM('Collection Curves'!D2:D6)</f>
+        <v>321.45</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -860,7 +887,31 @@
         <v>12</v>
       </c>
       <c r="B11" s="1">
-        <f>B8+B10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="1">
+        <v>15911.29</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="1">
+        <f>SUM('Recovery Analysis'!D2:D6)</f>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="1">
+        <f>B9+B13</f>
       </c>
     </row>
   </sheetData>
@@ -879,50 +930,50 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B4" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -943,30 +994,30 @@
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B2" s="1">
         <v>53527.04</v>
@@ -978,18 +1029,18 @@
         <f>B2-C2</f>
       </c>
       <c r="E2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B3" s="1">
         <v>53205.59</v>
@@ -1001,18 +1052,18 @@
         <f>B3-C3</f>
       </c>
       <c r="E3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B4" s="1">
         <v>15911.29</v>
@@ -1024,13 +1075,13 @@
         <f>B4-C4</f>
       </c>
       <c r="E4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F4" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G4" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -1049,72 +1100,72 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D4" t="s">
         <v>90</v>
-      </c>
-      <c r="B4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D4" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="C5" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="D5" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1125,7 +1176,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="18" customWidth="1"/>
@@ -1133,138 +1184,155 @@
   <sheetData>
     <row r="1" spans="1:5" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C2" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="D2" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E2" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="C3" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D3" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="E3" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B4" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C4" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="D4" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B5" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C5" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="D5" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E5" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B6" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C6" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D6" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="E6" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C7" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D7" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B8" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C8" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="D8" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="E8" t="s">
-        <v>43</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" t="s">
+        <v>127</v>
+      </c>
+      <c r="C9" t="s">
+        <v>128</v>
+      </c>
+      <c r="D9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E9" t="s">
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1287,7 +1355,7 @@
         <v>5</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1308,23 +1376,23 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B4" s="1">
-        <f>'Executive Summary'!B8</f>
+        <f>'Executive Summary'!B9</f>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1">
-        <f>'Executive Summary'!B10</f>
+        <f>'Executive Summary'!B13</f>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B6" s="1">
         <f>B4+B5</f>
@@ -1347,39 +1415,39 @@
   <sheetData>
     <row r="1" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>16</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="F2" s="1">
         <v>50000</v>
@@ -1387,19 +1455,19 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="s">
         <v>25</v>
       </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="F3" s="1">
         <v>3205.59</v>
@@ -1407,19 +1475,19 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="F4" s="1">
         <v>321.45</v>
@@ -1443,71 +1511,71 @@
   <sheetData>
     <row r="1" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F2" s="1">
         <v>6889.77</v>
       </c>
       <c r="G2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C3" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E3" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F3" s="1">
         <v>9021.52</v>
       </c>
       <c r="G3" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1527,15 +1595,15 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B2" s="1">
         <v>50000</v>
@@ -1543,7 +1611,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B3" s="1">
         <v>3205.59</v>
@@ -1566,7 +1634,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>7</v>
@@ -1574,7 +1642,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B2" s="1">
         <v>60000</v>
@@ -1582,7 +1650,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B3" s="1">
         <v>49646.56</v>
@@ -1605,7 +1673,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>7</v>
@@ -1613,7 +1681,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B2" s="1">
         <v>60000</v>
@@ -1621,7 +1689,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B3" s="1">
         <v>49646.56</v>
@@ -1644,7 +1712,7 @@
   <sheetData>
     <row r="1" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>7</v>
@@ -1652,7 +1720,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B2" s="1">
         <v>60000</v>
@@ -1660,7 +1728,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B3" s="1">
         <v>49646.56</v>
@@ -1684,21 +1752,21 @@
   <sheetData>
     <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B2" s="4">
         <v>0.9</v>
@@ -1712,7 +1780,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B3" s="4">
         <v>0.7</v>
@@ -1726,7 +1794,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B4" s="4">
         <v>0.5</v>
@@ -1740,7 +1808,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B5" s="4">
         <v>0.3</v>
@@ -1754,7 +1822,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B6" s="4">
         <v>0.1</v>

</xml_diff>